<commit_message>
corrected LPG ship with LPG properties and recalculated capacity penalty
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-ships.xlsx
+++ b/premise/data/additional_inventories/lci-ships.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/Github/premise/premise/data/additional_inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF4F689-4E17-1741-A45E-48F2FB1E57CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79BDFBC-15F6-A849-92C7-44ACDC21BD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20240" yWindow="720" windowWidth="22420" windowHeight="23000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="inventories" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="200">
   <si>
     <t>Database</t>
   </si>
@@ -627,6 +627,15 @@
   </si>
   <si>
     <t>80% reduction relative to using HFO at 75% engine load, according to Petzold et al., 2011, dx.doi.org/10.1021/es2021439</t>
+  </si>
+  <si>
+    <t>LPG (propane and butane)</t>
+  </si>
+  <si>
+    <t>26--27</t>
+  </si>
+  <si>
+    <t>9% penalty of load carrying capacity, due to the low gravimetric density of LPG.</t>
   </si>
 </sst>
 </file>
@@ -634,11 +643,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -701,7 +710,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
@@ -709,12 +718,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -723,17 +732,17 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -3759,8 +3768,8 @@
         <v>93</v>
       </c>
       <c r="B156" s="11">
-        <f>parameters!N9</f>
-        <v>158400000000</v>
+        <f>parameters!N11</f>
+        <v>163923092656.98508</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.2">
@@ -3768,8 +3777,8 @@
         <v>94</v>
       </c>
       <c r="B157" s="11">
-        <f>parameters!O9</f>
-        <v>153000000000</v>
+        <f>parameters!O11</f>
+        <v>159903865821.23132</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.2">
@@ -3777,8 +3786,8 @@
         <v>95</v>
       </c>
       <c r="B158" s="11">
-        <f>parameters!P9</f>
-        <v>162000000000</v>
+        <f>parameters!P11</f>
+        <v>166602577214.15421</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.2">
@@ -3786,8 +3795,8 @@
         <v>156</v>
       </c>
       <c r="B159" s="13">
-        <f>parameters!I9</f>
-        <v>0.12</v>
+        <f>parameters!I11</f>
+        <v>8.9316151905638519E-2</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.2">
@@ -3795,8 +3804,8 @@
         <v>157</v>
       </c>
       <c r="B160" s="13">
-        <f>parameters!J9</f>
-        <v>0.1</v>
+        <f>parameters!J11</f>
+        <v>7.4430126588032122E-2</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.2">
@@ -3804,8 +3813,8 @@
         <v>158</v>
       </c>
       <c r="B161" s="13">
-        <f>parameters!K9</f>
-        <v>0.15</v>
+        <f>parameters!K11</f>
+        <v>0.11164518988204816</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.2">
@@ -3822,7 +3831,7 @@
         <v>131</v>
       </c>
       <c r="B163" s="13">
-        <f>parameters!C20</f>
+        <f>parameters!C23</f>
         <v>0.49342105263157898</v>
       </c>
     </row>
@@ -3831,7 +3840,7 @@
         <v>132</v>
       </c>
       <c r="B164" s="13">
-        <f>parameters!D20</f>
+        <f>parameters!D23</f>
         <v>0.44407894736842107</v>
       </c>
     </row>
@@ -3840,7 +3849,7 @@
         <v>133</v>
       </c>
       <c r="B165" s="13">
-        <f>parameters!E20</f>
+        <f>parameters!E23</f>
         <v>0.54276315789473695</v>
       </c>
     </row>
@@ -3916,7 +3925,7 @@
       </c>
       <c r="B169" s="12">
         <f>0.11*(B162/B163)/46/(1-B159)</f>
-        <v>2.3405797101449274E-3</v>
+        <v>2.261718102541901E-3</v>
       </c>
       <c r="C169" t="s">
         <v>5</v>
@@ -3938,15 +3947,15 @@
       </c>
       <c r="J169">
         <f>B169</f>
-        <v>2.3405797101449274E-3</v>
+        <v>2.261718102541901E-3</v>
       </c>
       <c r="K169" s="6">
         <f>0.11*(B162/B165)/46/(1-B160)</f>
-        <v>2.080515297906602E-3</v>
+        <v>2.0230388022607075E-3</v>
       </c>
       <c r="L169" s="6">
         <f>0.11*(B162/B164)/46/(1-B161)</f>
-        <v>2.6924315619967797E-3</v>
+        <v>2.5761855529249592E-3</v>
       </c>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.2">
@@ -3955,7 +3964,7 @@
       </c>
       <c r="B170" s="11">
         <f>1/B156</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="C170" t="s">
         <v>19</v>
@@ -3970,22 +3979,22 @@
         <v>43</v>
       </c>
       <c r="H170" t="s">
-        <v>119</v>
+        <v>199</v>
       </c>
       <c r="I170">
         <v>5</v>
       </c>
       <c r="J170" s="11">
         <f>B170</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="K170" s="11">
         <f>1/B158</f>
-        <v>6.1728395061728393E-12</v>
+        <v>6.0023081078426567E-12</v>
       </c>
       <c r="L170" s="11">
         <f>1/B157</f>
-        <v>6.5359477124183003E-12</v>
+        <v>6.25375749900866E-12</v>
       </c>
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.2">
@@ -3994,7 +4003,7 @@
       </c>
       <c r="B171" s="11">
         <f>1/B156</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="C171" t="s">
         <v>19</v>
@@ -4009,22 +4018,22 @@
         <v>49</v>
       </c>
       <c r="H171" t="s">
-        <v>119</v>
+        <v>199</v>
       </c>
       <c r="I171">
         <v>5</v>
       </c>
       <c r="J171" s="11">
         <f>B171</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="K171" s="11">
         <f>1/B158</f>
-        <v>6.1728395061728393E-12</v>
+        <v>6.0023081078426567E-12</v>
       </c>
       <c r="L171" s="11">
         <f>1/B157</f>
-        <v>6.5359477124183003E-12</v>
+        <v>6.25375749900866E-12</v>
       </c>
     </row>
     <row r="172" spans="1:12" x14ac:dyDescent="0.2">
@@ -4057,7 +4066,7 @@
       </c>
       <c r="B173" s="12">
         <f>B169*3</f>
-        <v>7.0217391304347818E-3</v>
+        <v>6.7851543076257025E-3</v>
       </c>
       <c r="D173" t="s">
         <v>23</v>
@@ -4076,15 +4085,15 @@
       </c>
       <c r="J173" s="6">
         <f>B173</f>
-        <v>7.0217391304347818E-3</v>
+        <v>6.7851543076257025E-3</v>
       </c>
       <c r="K173" s="6">
         <f>K169*3</f>
-        <v>6.2415458937198059E-3</v>
+        <v>6.069116406782123E-3</v>
       </c>
       <c r="L173" s="6">
         <f>L169*3</f>
-        <v>8.0772946859903397E-3</v>
+        <v>7.7285566587748777E-3</v>
       </c>
     </row>
     <row r="174" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4093,7 +4102,7 @@
       </c>
       <c r="B174" s="11">
         <f>0.00186*(B169*46*B163/3.6)</f>
-        <v>2.7447916666666669E-5</v>
+        <v>2.6523108669611446E-5</v>
       </c>
       <c r="D174" t="s">
         <v>23</v>
@@ -4112,15 +4121,15 @@
       </c>
       <c r="J174" s="6">
         <f t="shared" ref="J174:J180" si="6">B174</f>
-        <v>2.7447916666666669E-5</v>
+        <v>2.6523108669611446E-5</v>
       </c>
       <c r="K174" s="6">
         <f>0.00186*(B169*46*B164/3.6)</f>
-        <v>2.4703125000000002E-5</v>
+        <v>2.3870797802650298E-5</v>
       </c>
       <c r="L174" s="6">
         <f>0.00186*(B169*46*B165/3.6)</f>
-        <v>3.0192708333333338E-5</v>
+        <v>2.9175419536572591E-5</v>
       </c>
     </row>
     <row r="175" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4129,7 +4138,7 @@
       </c>
       <c r="B175">
         <f>0.00117*(B169*46*B163/3.6)</f>
-        <v>1.7265625000000001E-5</v>
+        <v>1.6683890937336232E-5</v>
       </c>
       <c r="D175" t="s">
         <v>23</v>
@@ -4148,15 +4157,15 @@
       </c>
       <c r="J175" s="6">
         <f t="shared" si="6"/>
-        <v>1.7265625000000001E-5</v>
+        <v>1.6683890937336232E-5</v>
       </c>
       <c r="K175" s="6">
         <f>0.00117*(B169*46*B164/3.6)</f>
-        <v>1.5539062499999999E-5</v>
+        <v>1.5015501843602608E-5</v>
       </c>
       <c r="L175" s="6">
         <f>0.00117*(B169*46*B165/3.6)</f>
-        <v>1.8992187500000003E-5</v>
+        <v>1.8352280031069855E-5</v>
       </c>
     </row>
     <row r="176" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4165,7 +4174,7 @@
       </c>
       <c r="B176" s="11">
         <f>0.00003*(B169*46*B163/3.6)</f>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="D176" t="s">
         <v>23</v>
@@ -4184,15 +4193,15 @@
       </c>
       <c r="J176" s="6">
         <f t="shared" si="6"/>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="K176" s="6">
         <f>0.00003*(B169*46*B164/3.6)</f>
-        <v>3.984375E-7</v>
+        <v>3.8501286778468222E-7</v>
       </c>
       <c r="L176" s="6">
         <f>0.00003*(B169*46*B165/3.6)</f>
-        <v>4.8697916666666668E-7</v>
+        <v>4.7057128284794499E-7</v>
       </c>
     </row>
     <row r="177" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4201,7 +4210,7 @@
       </c>
       <c r="B177" s="11">
         <f>0.00003*(B169*46*B163/3.6)</f>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="D177" t="s">
         <v>23</v>
@@ -4220,15 +4229,15 @@
       </c>
       <c r="J177" s="6">
         <f t="shared" si="6"/>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="K177" s="6">
         <f>0.00003*(B169*46*B164/3.6)</f>
-        <v>3.984375E-7</v>
+        <v>3.8501286778468222E-7</v>
       </c>
       <c r="L177" s="6">
         <f>0.00003*(B169*46*B165/3.6)</f>
-        <v>4.8697916666666668E-7</v>
+        <v>4.7057128284794499E-7</v>
       </c>
     </row>
     <row r="178" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4237,7 +4246,7 @@
       </c>
       <c r="B178" s="11">
         <f>B169*0.02</f>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="D178" t="s">
         <v>23</v>
@@ -4256,15 +4265,15 @@
       </c>
       <c r="J178" s="6">
         <f t="shared" si="6"/>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="K178" s="6">
         <f>J178</f>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="L178" s="6">
         <f>0.067*B169</f>
-        <v>1.5681884057971014E-4</v>
+        <v>1.5153511287030737E-4</v>
       </c>
     </row>
     <row r="179" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4273,7 +4282,7 @@
       </c>
       <c r="B179" s="11">
         <f>0.00038*(B169*46*B163/3.6)</f>
-        <v>5.607638888888889E-6</v>
+        <v>5.4186996206733058E-6</v>
       </c>
       <c r="D179" t="s">
         <v>23</v>
@@ -4292,15 +4301,15 @@
       </c>
       <c r="J179" s="6">
         <f t="shared" si="6"/>
-        <v>5.607638888888889E-6</v>
+        <v>5.4186996206733058E-6</v>
       </c>
       <c r="K179" s="6">
         <f>0.00038*(B169*46*B164/3.6)</f>
-        <v>5.0468749999999999E-6</v>
+        <v>4.8768296586059753E-6</v>
       </c>
       <c r="L179" s="6">
         <f>0.00038*(B169*46*B165/3.6)</f>
-        <v>6.168402777777779E-6</v>
+        <v>5.9605695827406364E-6</v>
       </c>
     </row>
     <row r="180" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4309,7 +4318,7 @@
       </c>
       <c r="B180" s="11">
         <f>0.00002*(B169*46*B163/3.6)</f>
-        <v>2.9513888888888889E-7</v>
+        <v>2.8519471687754242E-7</v>
       </c>
       <c r="D180" t="s">
         <v>23</v>
@@ -4328,15 +4337,15 @@
       </c>
       <c r="J180" s="6">
         <f t="shared" si="6"/>
-        <v>2.9513888888888889E-7</v>
+        <v>2.8519471687754242E-7</v>
       </c>
       <c r="K180" s="11">
         <f>0.00002*(B169*46*B164/3.6)</f>
-        <v>2.65625E-7</v>
+        <v>2.5667524518978816E-7</v>
       </c>
       <c r="L180">
         <f>0.00002*(B169*46*B165/3.6)</f>
-        <v>3.2465277777777784E-7</v>
+        <v>3.1371418856529668E-7</v>
       </c>
     </row>
     <row r="182" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -6064,7 +6073,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F1A7F4-A2B5-7747-AA61-2990069064F9}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.1640625" bestFit="1" customWidth="1"/>
@@ -6195,14 +6204,14 @@
         <v>0.43880000000000002</v>
       </c>
       <c r="E5" s="16">
-        <f t="shared" ref="E5:E10" si="0">1/D5</f>
+        <f t="shared" ref="E5:E11" si="0">1/D5</f>
         <v>2.2789425706472195</v>
       </c>
       <c r="F5" s="16">
         <v>1.1000000000000001</v>
       </c>
       <c r="G5" s="16">
-        <f t="shared" ref="G5:G10" si="1">E5*F5</f>
+        <f t="shared" ref="G5:G11" si="1">E5*F5</f>
         <v>2.5068368277119415</v>
       </c>
       <c r="H5" s="14">
@@ -6422,7 +6431,7 @@
         <v>1.8000327278677795</v>
       </c>
       <c r="H9" s="14">
-        <f t="shared" si="2"/>
+        <f>1-(1/G9)</f>
         <v>0.44445454545454544</v>
       </c>
       <c r="I9" s="13">
@@ -6506,6 +6515,63 @@
         <v>117000000000</v>
       </c>
     </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" s="16">
+        <f>26.5/36</f>
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="E11" s="16">
+        <f t="shared" si="0"/>
+        <v>1.3584905660377358</v>
+      </c>
+      <c r="F11" s="16">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G11" s="16">
+        <f t="shared" si="1"/>
+        <v>1.4943396226415095</v>
+      </c>
+      <c r="H11" s="14">
+        <f>1-(1/G11)</f>
+        <v>0.33080808080808088</v>
+      </c>
+      <c r="I11" s="13">
+        <f>I9*H11/H9</f>
+        <v>8.9316151905638519E-2</v>
+      </c>
+      <c r="J11" s="13">
+        <f>J9*H11/H9</f>
+        <v>7.4430126588032122E-2</v>
+      </c>
+      <c r="K11" s="13">
+        <f>K9*H11/H9</f>
+        <v>0.11164518988204816</v>
+      </c>
+      <c r="L11" s="15">
+        <v>7200000000</v>
+      </c>
+      <c r="M11">
+        <v>25</v>
+      </c>
+      <c r="N11" s="15">
+        <f t="shared" ref="N11" si="8">L11*M11*(1-I11)</f>
+        <v>163923092656.98508</v>
+      </c>
+      <c r="O11" s="15">
+        <f t="shared" ref="O11" si="9">L11*M11*(1-K11)</f>
+        <v>159903865821.23132</v>
+      </c>
+      <c r="P11" s="15">
+        <f t="shared" ref="P11" si="10">L11*M11*(1-J11)</f>
+        <v>166602577214.15421</v>
+      </c>
+    </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="O12" s="11"/>
     </row>
@@ -6653,6 +6719,23 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
+        <v>197</v>
+      </c>
+      <c r="C23" s="14">
+        <f>3.6/(0.152*48)</f>
+        <v>0.49342105263157898</v>
+      </c>
+      <c r="D23" s="14">
+        <f>C23*0.9</f>
+        <v>0.44407894736842107</v>
+      </c>
+      <c r="E23" s="14">
+        <f>C23*1.1</f>
+        <v>0.54276315789473695</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
         <v>183</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added dataanalysis for hydrogen use in sectors
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-ships.xlsx
+++ b/premise/data/additional_inventories/lci-ships.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA23D2A4-BEA8-4936-BBFE-826CDCD39D6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B79077-8F25-4DC2-B2E2-0B7C8F7DAEBC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10500" yWindow="660" windowWidth="25824" windowHeight="18984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2490,8 +2490,8 @@
         <v>4.5451388888888888E-8</v>
       </c>
       <c r="K84" s="6">
-        <f t="shared" ref="K84:K86" si="2">0.00002*(B77*18.6*B72/3.6)</f>
-        <v>1.6145833333333334E-12</v>
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L84" s="6">
         <f>0.0000028*(B76*18.6*B72/3.6)</f>
@@ -2526,8 +2526,8 @@
         <v>6.4930555555555568E-7</v>
       </c>
       <c r="K85" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L85" s="6">
         <f>0.00004*(B76*18.6*B72/3.6)</f>
@@ -2561,9 +2561,9 @@
         <f t="shared" si="1"/>
         <v>7.4670138888888891E-7</v>
       </c>
-      <c r="K86" s="6" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
+      <c r="K86" s="6">
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L86">
         <f>0.00013*(B76*18.6*B72/3.6)</f>
@@ -2979,7 +2979,7 @@
         <v>5</v>
       </c>
       <c r="J112" s="6">
-        <f t="shared" ref="J112:J115" si="3">B112</f>
+        <f t="shared" ref="J112:J115" si="2">B112</f>
         <v>7.7916666666666672E-5</v>
       </c>
       <c r="K112" s="6">
@@ -3015,7 +3015,7 @@
         <v>5</v>
       </c>
       <c r="J113" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.3613953124999986E-5</v>
       </c>
       <c r="K113" s="6">
@@ -3051,7 +3051,7 @@
         <v>5</v>
       </c>
       <c r="J114" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.2035554687499993E-5</v>
       </c>
       <c r="K114" s="6">
@@ -3087,7 +3087,7 @@
         <v>5</v>
       </c>
       <c r="J115" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>7.953993055555555E-9</v>
       </c>
       <c r="K115" s="6">
@@ -3509,7 +3509,7 @@
         <v>5</v>
       </c>
       <c r="J141" s="6">
-        <f t="shared" ref="J141:J144" si="4">B141</f>
+        <f t="shared" ref="J141:J144" si="3">B141</f>
         <v>4.0680701754385975E-5</v>
       </c>
       <c r="K141" s="6">
@@ -3545,7 +3545,7 @@
         <v>5</v>
       </c>
       <c r="J142" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.5589473684210534E-5</v>
       </c>
       <c r="K142" s="6">
@@ -3581,7 +3581,7 @@
         <v>5</v>
       </c>
       <c r="J143" s="6">
-        <f t="shared" ref="J143" si="5">B143</f>
+        <f t="shared" ref="J143" si="4">B143</f>
         <v>6.5614035087719314E-7</v>
       </c>
       <c r="K143" s="6">
@@ -3617,7 +3617,7 @@
         <v>5</v>
       </c>
       <c r="J144" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>6.5614035087719314E-7</v>
       </c>
       <c r="K144" s="6">
@@ -3653,7 +3653,7 @@
         <v>5</v>
       </c>
       <c r="J145" s="6">
-        <f t="shared" ref="J145:J147" si="6">B145</f>
+        <f t="shared" ref="J145:J147" si="5">B145</f>
         <v>6.6488888888888891E-5</v>
       </c>
       <c r="K145" s="6">
@@ -3689,7 +3689,7 @@
         <v>5</v>
       </c>
       <c r="J146" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>8.311111111111113E-6</v>
       </c>
       <c r="K146" s="6">
@@ -3725,7 +3725,7 @@
         <v>5</v>
       </c>
       <c r="J147" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>4.3742690058479546E-7</v>
       </c>
       <c r="K147" s="11">
@@ -4142,7 +4142,7 @@
         <v>5</v>
       </c>
       <c r="J174" s="6">
-        <f t="shared" ref="J174:J180" si="7">B174</f>
+        <f t="shared" ref="J174:J180" si="6">B174</f>
         <v>2.6523108669611446E-5</v>
       </c>
       <c r="K174" s="6">
@@ -4178,7 +4178,7 @@
         <v>5</v>
       </c>
       <c r="J175" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.6683890937336232E-5</v>
       </c>
       <c r="K175" s="6">
@@ -4214,7 +4214,7 @@
         <v>5</v>
       </c>
       <c r="J176" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.2779207531631361E-7</v>
       </c>
       <c r="K176" s="6">
@@ -4250,7 +4250,7 @@
         <v>5</v>
       </c>
       <c r="J177" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.2779207531631361E-7</v>
       </c>
       <c r="K177" s="6">
@@ -4286,7 +4286,7 @@
         <v>5</v>
       </c>
       <c r="J178" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.5234362050838021E-5</v>
       </c>
       <c r="K178" s="6">
@@ -4322,7 +4322,7 @@
         <v>5</v>
       </c>
       <c r="J179" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>5.4186996206733058E-6</v>
       </c>
       <c r="K179" s="6">
@@ -4358,7 +4358,7 @@
         <v>5</v>
       </c>
       <c r="J180" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2.8519471687754242E-7</v>
       </c>
       <c r="K180" s="11">
@@ -4748,7 +4748,7 @@
         <v>5</v>
       </c>
       <c r="J206" s="6">
-        <f t="shared" ref="J206" si="8">B206</f>
+        <f t="shared" ref="J206" si="7">B206</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K206" s="6">
@@ -4784,7 +4784,7 @@
         <v>5</v>
       </c>
       <c r="J207" s="6">
-        <f t="shared" ref="J207:J211" si="9">B207</f>
+        <f t="shared" ref="J207:J211" si="8">B207</f>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K207" s="6">
@@ -4820,7 +4820,7 @@
         <v>5</v>
       </c>
       <c r="J208" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K208" s="6">
@@ -4856,7 +4856,7 @@
         <v>5</v>
       </c>
       <c r="J209" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K209" s="6">
@@ -4892,7 +4892,7 @@
         <v>5</v>
       </c>
       <c r="J210" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K210" s="6">
@@ -4928,7 +4928,7 @@
         <v>5</v>
       </c>
       <c r="J211" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K211" s="6">
@@ -5321,7 +5321,7 @@
         <v>5</v>
       </c>
       <c r="J237" s="6">
-        <f t="shared" ref="J237:J242" si="10">B237</f>
+        <f t="shared" ref="J237:J242" si="9">B237</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K237" s="6">
@@ -5357,7 +5357,7 @@
         <v>5</v>
       </c>
       <c r="J238" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K238" s="6">
@@ -5393,7 +5393,7 @@
         <v>5</v>
       </c>
       <c r="J239" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K239" s="6">
@@ -5429,7 +5429,7 @@
         <v>5</v>
       </c>
       <c r="J240" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K240" s="6">
@@ -5465,7 +5465,7 @@
         <v>5</v>
       </c>
       <c r="J241" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K241" s="6">
@@ -5501,7 +5501,7 @@
         <v>5</v>
       </c>
       <c r="J242" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K242" s="6">
@@ -5894,7 +5894,7 @@
         <v>5</v>
       </c>
       <c r="J268" s="6">
-        <f t="shared" ref="J268:J273" si="11">B268</f>
+        <f t="shared" ref="J268:J273" si="10">B268</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K268" s="6">
@@ -5930,7 +5930,7 @@
         <v>5</v>
       </c>
       <c r="J269" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K269" s="6">
@@ -5966,7 +5966,7 @@
         <v>5</v>
       </c>
       <c r="J270" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K270" s="6">
@@ -6002,7 +6002,7 @@
         <v>5</v>
       </c>
       <c r="J271" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K271" s="6">
@@ -6038,7 +6038,7 @@
         <v>5</v>
       </c>
       <c r="J272" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K272" s="6">
@@ -6074,7 +6074,7 @@
         <v>5</v>
       </c>
       <c r="J273" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K273" s="6">

</xml_diff>